<commit_message>
RESHIPPED (task266): asks re-cut with silent primaries under the policy's pins, the call frozen
The wave 3 audit found the round-1 fix had filed every ask device in the
registrar's notes, so a solver executing the notes hit all eighteen ask
figures. The notes are back to flat field definitions. Underneath the
pins now sit the extract's course credit hours (linked sections, and two
gateway courses at their spring 2027 hours), late adds after the census,
and each program's accelerated eight-week pair sharing one instructor,
room and time. Every main-call figure is unchanged; judge pass 3
DETERMINISTIC and APPROVE.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142Jt4Mt622iBfGoK24ivCU
</commit_message>
<xml_diff>
--- a/task266/golden/program_completion_review_2027.xlsx
+++ b/task266/golden/program_completion_review_2027.xlsx
@@ -131,7 +131,7 @@
     <t>Students who died (5) are removed from the classes. FTE and classes are the review profile of Policy 3.12, section 4.</t>
   </si>
   <si>
-    <t>77 of Nursing's 78 classes under ten are clinical groups, which take at most eight students each.</t>
+    <t>77 of Nursing's 79 classes under ten are clinical groups, which take at most eight students each.</t>
   </si>
   <si>
     <t>Term since entry</t>
@@ -161,10 +161,10 @@
     <t>The fall 2024 class is observed to its eighth term and the fall 2025 class to its fifth; their later terms use the rates of the classes observed in those terms.</t>
   </si>
   <si>
-    <t>FTE: credit hours registered at the fall 2026 census (registrations in place on 8 September 2026, later withdrawals included), each course counted at its section credit hours (laboratory, shop and clinical sections carry none), by each student's program of record for fall 2026, divided by 15.</t>
-  </si>
-  <si>
-    <t>Classes under ten students: sections of each program's own subjects that ran in fall 2026, sections taught together at one meeting (interactive video between campuses) counted as one class with their students added; census registrations as above.</t>
+    <t>FTE: credit hours registered at the fall 2026 census (registrations in place on 8 September 2026, later withdrawals included and registrations added after that date not), each at its section's credit hours in the fall 2026 schedule (laboratory, shop and clinical sections carry none, and English Composition I and College Algebra ran at three), by each student's program of record for fall 2026, divided by 15.</t>
+  </si>
+  <si>
+    <t>Classes under ten students: sections of each program's own subjects that ran in fall 2026, sections taught together at one meeting (interactive video between campuses) counted as one class with their students added; the accelerated sections that share a room and time in the first and second eight weeks are two classes; census registrations as above.</t>
   </si>
   <si>
     <t>Shares are rounded to one decimal place from the unrounded estimate; the floor is applied to the unrounded share.</t>
@@ -671,10 +671,10 @@
         <v>13</v>
       </c>
       <c r="G5" s="7">
-        <v>1164.1</v>
+        <v>1148.8</v>
       </c>
       <c r="H5" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -697,10 +697,10 @@
         <v>13</v>
       </c>
       <c r="G6" s="7">
-        <v>358</v>
+        <v>352.5</v>
       </c>
       <c r="H6" s="8">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -723,10 +723,10 @@
         <v>13</v>
       </c>
       <c r="G7" s="7">
-        <v>531.7</v>
+        <v>525.2</v>
       </c>
       <c r="H7" s="8">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -749,10 +749,10 @@
         <v>13</v>
       </c>
       <c r="G8" s="7">
-        <v>404</v>
+        <v>399.4</v>
       </c>
       <c r="H8" s="8">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -775,10 +775,10 @@
         <v>13</v>
       </c>
       <c r="G9" s="7">
-        <v>386.6</v>
+        <v>381.5</v>
       </c>
       <c r="H9" s="8">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -801,10 +801,10 @@
         <v>13</v>
       </c>
       <c r="G10" s="7">
-        <v>343.6</v>
+        <v>341</v>
       </c>
       <c r="H10" s="8">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -827,10 +827,10 @@
         <v>28</v>
       </c>
       <c r="G11" s="7">
-        <v>397.1</v>
+        <v>391.2</v>
       </c>
       <c r="H11" s="8">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -853,10 +853,10 @@
         <v>28</v>
       </c>
       <c r="G12" s="7">
-        <v>274.5</v>
+        <v>272.3</v>
       </c>
       <c r="H12" s="8">
-        <v>13</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -879,10 +879,10 @@
         <v>28</v>
       </c>
       <c r="G13" s="7">
-        <v>538.3</v>
+        <v>533.1</v>
       </c>
       <c r="H13" s="8">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>